<commit_message>
Use hugepages for benchmark runs
</commit_message>
<xml_diff>
--- a/tests/FlowTable_Test_Cases.xlsx
+++ b/tests/FlowTable_Test_Cases.xlsx
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">8.08 Mpps</t>
+          <t xml:space="preserve">21.28 Mpps</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">i5-8250U; no hugepages; synthetic flow engine</t>
+          <t xml:space="preserve">i5-8250U; hugepages; synthetic flow engine</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1116,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.78x / 14.34 Mpps</t>
+          <t xml:space="preserve">1.95x / 41.44 Mpps</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.49x / 20.08 Mpps</t>
+          <t xml:space="preserve">2.69x / 57.23 Mpps</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -1210,7 +1210,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">9.77 / 17.32 / 22.88 Mpps</t>
+          <t xml:space="preserve">22.51 / 45.62 / 66.66 Mpps</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1M packets, 100k bidirectional flows</t>
+          <t xml:space="preserve">200k packets, 100k generated SPI flows</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1252,12 +1252,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">See README run command</t>
+          <t xml:space="preserve">make benchmark-e2e</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.84 Mpps median; zero loss</t>
+          <t xml:space="preserve">1.57 Mpps PCAP PMD; zero loss</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Untagged subnet resolver; single dispatcher plus four workers</t>
+          <t xml:space="preserve">Generated Ethernet PCAP from SPI_DPI_rule.xlsx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stabilize e2e benchmark runs
</commit_message>
<xml_diff>
--- a/tests/FlowTable_Test_Cases.xlsx
+++ b/tests/FlowTable_Test_Cases.xlsx
@@ -1237,7 +1237,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">200k packets, 100k generated SPI flows</t>
+          <t xml:space="preserve">1M packets, 100k generated SPI flows</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.02 Mpps single PCAP; 4.60 Mpps multi-RX PCAP; zero loss</t>
+          <t xml:space="preserve">1.95 Mpps single PCAP; 2.63 Mpps multi-RX PCAP; zero loss</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Generated Ethernet PCAP from SPI_DPI_rule.xlsx; 4 active workers</t>
+          <t xml:space="preserve">2 warmup + 5 measured runs; median PPS; 4 active workers</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use fixed multi-worker path for e2e pcap benchmark
</commit_message>
<xml_diff>
--- a/tests/FlowTable_Test_Cases.xlsx
+++ b/tests/FlowTable_Test_Cases.xlsx
@@ -1257,7 +1257,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.62 Mpps PCAP PMD; zero loss</t>
+          <t xml:space="preserve">3.17 Mpps PCAP PMD; zero loss</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Generated Ethernet PCAP from SPI_DPI_rule.xlsx</t>
+          <t xml:space="preserve">Generated Ethernet PCAP from SPI_DPI_rule.xlsx; 4 active workers</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Align pcap benchmark with infinite rx workload
</commit_message>
<xml_diff>
--- a/tests/FlowTable_Test_Cases.xlsx
+++ b/tests/FlowTable_Test_Cases.xlsx
@@ -1237,7 +1237,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1M packets, 100k generated SPI flows</t>
+          <t xml:space="preserve">200k packets, 100k generated SPI flows</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.95 Mpps single PCAP; 2.63 Mpps multi-RX PCAP; zero loss</t>
+          <t xml:space="preserve">3.14 Mpps single PCAP; 4.35 Mpps multi-RX PCAP; zero loss</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 warmup + 5 measured runs; median PPS; 4 active workers</t>
+          <t xml:space="preserve">infinite_rx=1; 2 warmup + 5 measured runs; median PPS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactor codes for project requirement, benchmarks and generate required diagrams
</commit_message>
<xml_diff>
--- a/tests/FlowTable_Test_Cases.xlsx
+++ b/tests/FlowTable_Test_Cases.xlsx
@@ -1257,7 +1257,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.46 Mpps single PCAP; 7.24 Mpps multi-RX PCAP; zero loss</t>
+          <t xml:space="preserve">5.46 Mpps single PCAP; 7.24 Mpps multi-RX PCAP; zero loss; 100k active flows</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">All packets create new flows</t>
+          <t xml:space="preserve">100k unique flows in E2E PCAP</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1294,27 +1294,27 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Establish server-specific baseline</t>
+          <t xml:space="preserve">Report create/delete rates</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Benchmark variant</t>
+          <t xml:space="preserve">make benchmark-e2e</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not measured</t>
+          <t xml:space="preserve">2.73 Mflows/s single PCAP; 3.62 Mflows/s multi-RX; delete/timeout=0/s</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NOT RUN</t>
+          <t xml:space="preserve">PASS</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Current CPU field is lcore allocation: 5/8 and 7/8 logical CPUs</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove synthetic path and split pipeline runtime
</commit_message>
<xml_diff>
--- a/tests/FlowTable_Test_Cases.xlsx
+++ b/tests/FlowTable_Test_Cases.xlsx
@@ -795,7 +795,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No packet loss in synthetic pipeline</t>
+          <t xml:space="preserve">No packet loss in PCAP PMD pipeline</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -805,12 +805,12 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Run 1,000,000 packets / 100,000 flows</t>
+          <t xml:space="preserve">Replay generated SPI PCAP</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">dispatched=processed=1,000,000</t>
+          <t xml:space="preserve">dispatched=processed and dropped=0</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recorded in reports/BENCHMARK.md</t>
+          <t xml:space="preserve">reports/e2e_benchmark_results.csv</t>
         </is>
       </c>
     </row>
@@ -1044,32 +1044,32 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">One-core baseline</t>
+          <t xml:space="preserve">Single-dispatcher E2E</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">32,768 flows/worker, 2M packets</t>
+          <t xml:space="preserve">200k packets, 100k generated SPI flows</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PPS</t>
+          <t xml:space="preserve">PPS and loss</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Record baseline</t>
+          <t xml:space="preserve">processed=dispatched; no unexpected drop</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">make benchmark</t>
+          <t xml:space="preserve">make benchmark-e2e</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">21.28 Mpps</t>
+          <t xml:space="preserve">5.46 Mpps; zero loss; 100k active flows</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">i5-8250U; hugepages; synthetic flow engine</t>
+          <t xml:space="preserve">infinite_rx=1; 2 warmup + 5 measured runs; median PPS</t>
         </is>
       </c>
     </row>
@@ -1091,32 +1091,32 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Two-core scale</t>
+          <t xml:space="preserve">Multi-RX E2E</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Same workload per worker</t>
+          <t xml:space="preserve">2 RX queues, 2 dispatchers, 4 workers</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scale-up</t>
+          <t xml:space="preserve">PPS and scale</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&gt;=1.6x on laptop; &gt;=1.8x on server</t>
+          <t xml:space="preserve">Outperform single-dispatcher profile</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">make benchmark</t>
+          <t xml:space="preserve">make benchmark-e2e</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1.95x / 41.44 Mpps</t>
+          <t xml:space="preserve">7.24 Mpps; 1.33x over single-dispatcher PCAP</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1126,7 +1126,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Independent sharded flow tables</t>
+          <t xml:space="preserve">PCAP PMD shards; --per-dispatcher-limit</t>
         </is>
       </c>
     </row>
@@ -1138,42 +1138,42 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Four-core scale</t>
+          <t xml:space="preserve">Flow creation rate</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Same workload per worker</t>
+          <t xml:space="preserve">100k unique flows in E2E PCAP</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Scale-up</t>
+          <t xml:space="preserve">Flows/s</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&gt;=2.2x on laptop; &gt;=3.2x production target</t>
+          <t xml:space="preserve">Report create/delete rates</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">make benchmark</t>
+          <t xml:space="preserve">make benchmark-e2e</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.69x / 57.23 Mpps</t>
+          <t xml:space="preserve">2.73 Mflows/s single PCAP; 3.62 Mflows/s multi-RX; delete/timeout=0/s</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">ENV-LIMITED</t>
+          <t xml:space="preserve">PASS</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Laptop turbo and shared LLC/memory limit linearity</t>
+          <t xml:space="preserve">Current CPU field is lcore allocation: 5/8 and 7/8 logical CPUs</t>
         </is>
       </c>
     </row>
@@ -1185,42 +1185,42 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hot-cache scale</t>
+          <t xml:space="preserve">Realtime CLI benchmark</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">4,096 flows/worker, 5M packets</t>
+          <t xml:space="preserve">PCAP PMD with infinite_rx=1</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PPS and scale</t>
+          <t xml:space="preserve">Live PPS/flows/drops</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Trend increases for 1/2/4 cores</t>
+          <t xml:space="preserve">CLI updates while pipeline is running</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">make benchmark</t>
+          <t xml:space="preserve">scripts/run_cli_pcap.sh then show benchmark</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">22.51 / 45.62 / 66.66 Mpps</t>
+          <t xml:space="preserve">Command implemented; manual visual check required</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">READY</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">show dashboard also renders Active Flow, Throughput, Packet Drop graphs</t>
         </is>
       </c>
     </row>
@@ -1232,42 +1232,42 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">End-to-end pipeline</t>
+          <t xml:space="preserve">Dashboard graphs</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">200k packets, 100k generated SPI flows</t>
+          <t xml:space="preserve">Running CLI or --dashboard mode</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PPS and loss</t>
+          <t xml:space="preserve">Graph visibility</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">processed=dispatched; no unexpected drop</t>
+          <t xml:space="preserve">Active Flow, Throughput and Packet Drop are rendered</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">make benchmark-e2e</t>
+          <t xml:space="preserve">show dashboard</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.46 Mpps single PCAP; 7.24 Mpps multi-RX PCAP; zero loss; 100k active flows</t>
+          <t xml:space="preserve">Implemented</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">READY</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">infinite_rx=1; 2 warmup + 5 measured runs; median PPS</t>
+          <t xml:space="preserve">ASCII history, 32 samples</t>
         </is>
       </c>
     </row>
@@ -1279,42 +1279,42 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flow creation rate</t>
+          <t xml:space="preserve">Aging pressure</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">100k unique flows in E2E PCAP</t>
+          <t xml:space="preserve">90% idle flows; timeout scan active</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Flows/s</t>
+          <t xml:space="preserve">PPS degradation</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Report create/delete rates</t>
+          <t xml:space="preserve">&lt;10% throughput loss</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">make benchmark-e2e</t>
+          <t xml:space="preserve">Run for &gt;5 seconds</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.73 Mflows/s single PCAP; 3.62 Mflows/s multi-RX; delete/timeout=0/s</t>
+          <t xml:space="preserve">Not measured</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PASS</t>
+          <t xml:space="preserve">NOT RUN</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Current CPU field is lcore allocation: 5/8 and 7/8 logical CPUs</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -1326,27 +1326,27 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Aging pressure</t>
+          <t xml:space="preserve">Ring backpressure</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">90% idle flows; timeout scan active</t>
+          <t xml:space="preserve">Bursty RX beyond worker service rate</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PPS degradation</t>
+          <t xml:space="preserve">Drop rate</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;10% throughput loss</t>
+          <t xml:space="preserve">No silent loss; counters reconcile</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Run for &gt;5 seconds</t>
+          <t xml:space="preserve">Traffic generator</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1373,42 +1373,42 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ring backpressure</t>
+          <t xml:space="preserve">NUMA locality</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bursty RX beyond worker service rate</t>
+          <t xml:space="preserve">Local vs remote allocation on 2-socket host</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drop rate</t>
+          <t xml:space="preserve">PPS/latency delta</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No silent loss; counters reconcile</t>
+          <t xml:space="preserve">Local allocation outperforms remote</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Traffic generator</t>
+          <t xml:space="preserve">Run with explicit lcore/socket maps</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Not measured</t>
+          <t xml:space="preserve">Host has one NUMA node</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NOT RUN</t>
+          <t xml:space="preserve">N/A</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Requires dual-socket server</t>
         </is>
       </c>
     </row>
@@ -1420,93 +1420,46 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">NUMA locality</t>
+          <t xml:space="preserve">PCAP PMD replay</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Local vs remote allocation on 2-socket host</t>
+          <t xml:space="preserve">Representative traffic.pcap</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PPS/latency delta</t>
+          <t xml:space="preserve">PPS/rule accuracy</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Local allocation outperforms remote</t>
+          <t xml:space="preserve">No parse errors; expected rule hits</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Run with explicit lcore/socket maps</t>
+          <t xml:space="preserve">--vdev net_pcap0 + --mode ethdev</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Host has one NUMA node</t>
+          <t xml:space="preserve">Not measured</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N/A</t>
+          <t xml:space="preserve">NOT RUN</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Requires dual-socket server</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PT-010</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PCAP PMD replay</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Representative traffic.pcap</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PPS/rule accuracy</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No parse errors; expected rule hits</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">--vdev net_pcap0 + --mode ethdev</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not measured</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">NOT RUN</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
           <t xml:space="preserve">Requires a supplied PCAP</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I11"/>
+  <autoFilter ref="A1:I10"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Make CLI dynamic scaling focused
</commit_message>
<xml_diff>
--- a/tests/FlowTable_Test_Cases.xlsx
+++ b/tests/FlowTable_Test_Cases.xlsx
@@ -1185,7 +1185,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Realtime CLI benchmark</t>
+          <t xml:space="preserve">Realtime CLI dynamic scaling</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1195,17 +1195,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Live PPS/flows/drops</t>
+          <t xml:space="preserve">Active worker control</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CLI updates while pipeline is running</t>
+          <t xml:space="preserve">scale up/down changes active worker count</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">scripts/run_cli_pcap.sh then show benchmark</t>
+          <t xml:space="preserve">scripts/run_cli_pcap.sh then scale up/down</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1220,7 +1220,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">show dashboard also renders Active Flow, Throughput, Packet Drop graphs</t>
+          <t xml:space="preserve">Default CLI mode starts workers=2 max-workers=4 without --fixed-workers</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Modify dynamic scaling validity, add more comments
</commit_message>
<xml_diff>
--- a/tests/FlowTable_Test_Cases.xlsx
+++ b/tests/FlowTable_Test_Cases.xlsx
@@ -1195,12 +1195,12 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Active worker control</t>
+          <t xml:space="preserve">Active worker rebalance</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">scale up/down changes active worker count</t>
+          <t xml:space="preserve">scale up/down changes active workers and flow placement</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1220,7 +1220,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Default CLI mode starts workers=2 max-workers=4 without --fixed-workers</t>
+          <t xml:space="preserve">Default CLI starts 2/4 workers; rebalance runs outside fixed-worker benchmark</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Matching test workbook and test cases with new benchmark
</commit_message>
<xml_diff>
--- a/tests/FlowTable_Test_Cases.xlsx
+++ b/tests/FlowTable_Test_Cases.xlsx
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">5.46 Mpps; zero loss; 100k active flows</t>
+          <t xml:space="preserve">6.43 Mpps; zero loss; 100k active flows</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -1116,7 +1116,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">7.24 Mpps; 1.33x over single-dispatcher PCAP</t>
+          <t xml:space="preserve">9.57 Mpps; 1.49x over single-dispatcher PCAP</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">2.73 Mflows/s single PCAP; 3.62 Mflows/s multi-RX; delete/timeout=0/s</t>
+          <t xml:space="preserve">3.22 Mflows/s single PCAP; 4.79 Mflows/s multi-RX; delete/timeout=0/s</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add new benchmark after run configuration
</commit_message>
<xml_diff>
--- a/tests/FlowTable_Test_Cases.xlsx
+++ b/tests/FlowTable_Test_Cases.xlsx
@@ -1049,7 +1049,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">200k packets, 100k generated SPI flows</t>
+          <t xml:space="preserve">2M processed packets, 100k generated SPI flows</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">6.43 Mpps; zero loss; 100k active flows</t>
+          <t xml:space="preserve">6.75 Mpps; zero loss; 100k active flows</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">infinite_rx=1; 2 warmup + 5 measured runs; median PPS</t>
+          <t xml:space="preserve">200k-packet base PCAP replayed by infinite_rx=1; 2 warmup + 5 measured runs; median PPS</t>
         </is>
       </c>
     </row>
@@ -1116,7 +1116,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">9.57 Mpps; 1.49x over single-dispatcher PCAP</t>
+          <t xml:space="preserve">10.26 Mpps; 1.52x over single-dispatcher PCAP</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1163,7 +1163,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3.22 Mflows/s single PCAP; 4.79 Mflows/s multi-RX; delete/timeout=0/s</t>
+          <t xml:space="preserve">0.34 Mflows/s single PCAP; 0.51 Mflows/s multi-RX; delete/timeout=0/s</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">

</xml_diff>